<commit_message>
Updated Lab Results and Survey Docs
</commit_message>
<xml_diff>
--- a/State lab test results/SDVL_Results.xlsx
+++ b/State lab test results/SDVL_Results.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alex/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alex/Documents/GitHub/BackyardBirds/State lab test results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CFA8C65-545A-F241-A7F3-2A31FCCCC789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C666E7E-A7E3-7F44-94A2-21B49A8FA758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3080" yWindow="2160" windowWidth="28040" windowHeight="17180" xr2:uid="{BE4D56C9-88CE-FE4C-A4D2-BDDE1F9C4E21}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Results" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="52">
   <si>
     <t>USGS#,Soil_ID</t>
   </si>
@@ -164,9 +164,6 @@
     <t>Pseudomonas alvei</t>
   </si>
   <si>
-    <t>3171-38516</t>
-  </si>
-  <si>
     <t>LEEBF-S3</t>
   </si>
   <si>
@@ -180,13 +177,28 @@
   </si>
   <si>
     <t>WEAGLECONPace-E</t>
+  </si>
+  <si>
+    <t>3171-38516-S2</t>
+  </si>
+  <si>
+    <t>Pseudomonas koreensis</t>
+  </si>
+  <si>
+    <t>Klebsiella aerogenes</t>
+  </si>
+  <si>
+    <t>Citrobacter freundii</t>
+  </si>
+  <si>
+    <t>Enterobacter sp.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -206,6 +218,12 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -252,12 +270,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1050,7 +1069,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B25" s="1">
         <v>45820</v>
@@ -1061,10 +1080,16 @@
       <c r="D25" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="E25" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B26" s="1">
         <v>45854</v>
@@ -1075,10 +1100,13 @@
       <c r="D26" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="E26" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B27" s="1">
         <v>45853</v>
@@ -1089,10 +1117,16 @@
       <c r="D27" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="E27" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B28" s="1">
         <v>45853</v>
@@ -1103,10 +1137,16 @@
       <c r="D28" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="E28" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B29" s="1">
         <v>45853</v>
@@ -1117,10 +1157,16 @@
       <c r="D29" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="E29" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B30" s="1">
         <v>45853</v>
@@ -1131,6 +1177,12 @@
       <c r="D30" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="E30" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C31" s="2" t="s">
@@ -1139,5 +1191,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>